<commit_message>
Update verified metadata extractions and identify historical outputs
</commit_message>
<xml_diff>
--- a/data/metadata_change.xlsx
+++ b/data/metadata_change.xlsx
@@ -1824,6 +1824,11 @@
       <c r="AD4" s="5" t="s">
         <v>40</v>
       </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Lohmann 2024 SI表S5为b=−0.018、SE=0.096。换算所用N需统一确认，本次未用候选值替换原零值。</t>
+        </is>
+      </c>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
@@ -1850,8 +1855,8 @@
       <c r="H5" s="5">
         <v>4</v>
       </c>
-      <c r="I5" s="6">
-        <v>-1E-4</v>
+      <c r="I5" s="6" t="n">
+        <v>-0.04491233209360376</v>
       </c>
       <c r="J5" s="7">
         <v>1449</v>
@@ -1901,20 +1906,23 @@
       <c r="Z5" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="AA5" s="5">
-        <v>1E-4</v>
+      <c r="AA5" s="5" t="n">
+        <v>0.04491233209360376</v>
       </c>
       <c r="AB5" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="AC5" s="5">
-        <v>2.8E-3</v>
+      <c r="AC5" s="5" t="n">
+        <v>0.002811079522297858</v>
       </c>
       <c r="AD5" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="AE5" s="5" t="s">
-        <v>66</v>
+      <c r="AE5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：已按Nowak 表1（PDF第12–13页）菜品碳排放值及销量频数修正。对照821单、标签628单，均值分别为4.087088916和3.986624204，样本SD为2.303624700和2.146525564。Cohensd=(标签均值−对照均值)/合并SD=−0.044912332094，direction=−1，cohens_d=0.044912332094，v=0.002811079522。SampleSize仍为1449。沿用原有两组SMD提取口径；本次算术修正不另行估计时期聚类方差。
+原记录（保留追溯）：pre-post examination</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.2">
@@ -2174,6 +2182,11 @@
       <c r="AD8" s="5" t="s">
         <v>65</v>
       </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Sun：现有d、v尚未追溯至一致的结局及转换输入，需补充SI或原提取工作纸。</t>
+        </is>
+      </c>
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
@@ -3598,6 +3611,11 @@
       <c r="AD24" s="5" t="s">
         <v>65</v>
       </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Casati：需确认原提取模型、比较对象及v来源，未以另一模型的候选值替换。</t>
+        </is>
+      </c>
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
@@ -3684,8 +3702,11 @@
       <c r="AC25" s="5">
         <v>1.2200000000000001E-2</v>
       </c>
-      <c r="AE25" s="5" t="s">
-        <v>148</v>
+      <c r="AE25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Nishino：243/126/120为组别×轮次的重复观测，需确认方差如何处理组内重复，不能仅更换N重算。
+原记录（保留追溯）：CFP labels are attached with one product under open information</t>
+        </is>
       </c>
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.2">
@@ -3773,8 +3794,11 @@
       <c r="AC26" s="5">
         <v>1.26E-2</v>
       </c>
-      <c r="AE26" s="5" t="s">
-        <v>149</v>
+      <c r="AE26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Nishino：243/126/120为组别×轮次的重复观测，需确认方差如何处理组内重复，不能仅更换N重算。
+原记录（保留追溯）：CFP labels are attached with two products under open information</t>
+        </is>
       </c>
     </row>
     <row r="27" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -3868,8 +3892,11 @@
       <c r="AD27" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AE27" s="1" t="s">
-        <v>162</v>
+      <c r="AE27" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Slapø：现有v可由51个对照时段及41个干预时段重建，与仅采用stage 1的原备注需核对，等待附录及时间窗确认。
+原记录（保留追溯）：这里的v采用了全局v，仅仅采纳了stage1干预</t>
+        </is>
       </c>
     </row>
     <row r="28" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -3963,8 +3990,11 @@
       <c r="AD28" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AE28" s="1" t="s">
-        <v>162</v>
+      <c r="AE28" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Slapø：现有v可由51个对照时段及42个干预时段重建，与仅采用stage 1的原备注需核对，等待附录及时间窗确认。
+原记录（保留追溯）：这里的v采用了全局v，仅仅采纳了stage1干预</t>
+        </is>
       </c>
     </row>
     <row r="29" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -4058,8 +4088,11 @@
       <c r="AD29" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AE29" s="1" t="s">
-        <v>162</v>
+      <c r="AE29" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Slapø：现有v可由51个对照时段及42个干预时段重建，与仅采用stage 1的原备注需核对，等待附录及时间窗确认。
+原记录（保留追溯）：这里的v采用了全局v，仅仅采纳了stage1干预</t>
+        </is>
       </c>
     </row>
     <row r="30" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -4301,14 +4334,14 @@
       <c r="X32" t="s">
         <v>263</v>
       </c>
-      <c r="Y32" s="5">
-        <v>1</v>
+      <c r="Y32" s="5" t="n">
+        <v>-1</v>
       </c>
       <c r="Z32" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="AA32" s="5">
-        <v>-7.9571439999999993E-3</v>
+      <c r="AA32" s="5" t="n">
+        <v>0.007957144</v>
       </c>
       <c r="AB32" s="5" t="s">
         <v>185</v>
@@ -4318,6 +4351,11 @@
       </c>
       <c r="AD32" s="5" t="s">
         <v>65</v>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：已修正。Engström 原文表3（PDF第6页）：高排放餐份额下降，按正值代表更低碳选择修正方向。 原始Cohensd、v及SampleSize保持不变。</t>
+        </is>
       </c>
     </row>
     <row r="33" spans="1:30" x14ac:dyDescent="0.2">
@@ -4405,6 +4443,11 @@
       <c r="AD33" s="5" t="s">
         <v>65</v>
       </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Engström 中排放类别的增减不能单独确定总体低碳方向，等待结局编码规则确认。</t>
+        </is>
+      </c>
     </row>
     <row r="34" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
@@ -4559,14 +4602,14 @@
       <c r="X35" t="s">
         <v>267</v>
       </c>
-      <c r="Y35" s="5">
-        <v>-1</v>
+      <c r="Y35" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="Z35" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="AA35" s="5">
-        <v>-0.29420000000000002</v>
+      <c r="AA35" s="5" t="n">
+        <v>0.2942</v>
       </c>
       <c r="AB35" s="5" t="s">
         <v>195</v>
@@ -4576,6 +4619,11 @@
       </c>
       <c r="AD35" s="5" t="s">
         <v>196</v>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：已修正。Cadario Study 4（PDF第7页）：动物性零食选择由32%降至19%，修正为有利方向。保留原转换方法及效应量幅度。 原始Cohensd、v及SampleSize保持不变。</t>
+        </is>
       </c>
     </row>
     <row r="36" spans="1:30" x14ac:dyDescent="0.2">
@@ -4749,6 +4797,11 @@
       <c r="AD37" s="5" t="s">
         <v>40</v>
       </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Jones 中排放类别的增减不能单独确定总体低碳方向，等待结局编码规则确认。</t>
+        </is>
+      </c>
     </row>
     <row r="38" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
@@ -4921,6 +4974,11 @@
       <c r="AD39" s="5" t="s">
         <v>65</v>
       </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。De Visser：现有值对应全部三明治总销量差异，需确认其结局纳入及按日分析口径。</t>
+        </is>
+      </c>
     </row>
     <row r="40" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
@@ -5007,6 +5065,11 @@
       <c r="AD40" s="5" t="s">
         <v>65</v>
       </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。De Visser：现有值来自总销售计数，需确认按日分析口径及local-only条件的纳入。</t>
+        </is>
+      </c>
     </row>
     <row r="41" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
@@ -5093,6 +5156,11 @@
       <c r="AD41" s="5" t="s">
         <v>65</v>
       </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。De Visser：现有值来自总销售计数，需补足按日标准化所需输入后再决定替换。</t>
+        </is>
+      </c>
     </row>
     <row r="42" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
@@ -5179,6 +5247,11 @@
       <c r="AD42" s="5" t="s">
         <v>65</v>
       </c>
+      <c r="AE42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。De Visser：现有值来自总销售计数，需补足按日标准化所需输入后再决定替换。</t>
+        </is>
+      </c>
     </row>
     <row r="43" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
@@ -5247,14 +5320,14 @@
       <c r="X43" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="Y43" s="1">
-        <v>1</v>
+      <c r="Y43" s="1" t="n">
+        <v>-1</v>
       </c>
       <c r="Z43" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="AA43" s="1">
-        <v>0.1575</v>
+      <c r="AA43" s="1" t="n">
+        <v>-0.1575</v>
       </c>
       <c r="AB43" s="1" t="s">
         <v>227</v>
@@ -5264,6 +5337,11 @@
       </c>
       <c r="AD43" s="1" t="s">
         <v>65</v>
+      </c>
+      <c r="AE43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：已修正。ElHaffar 表1–2（PDF第7页）：交通灯条件低排放菜日销量151.375低于对照164.875，修正为负向。 原始Cohensd、v及SampleSize保持不变。 沿用当前提取的绝对日销量结局，未改为销量份额。</t>
+        </is>
       </c>
     </row>
     <row r="44" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -5333,14 +5411,14 @@
       <c r="X44" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="Y44" s="1">
-        <v>-1</v>
+      <c r="Y44" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="Z44" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="AA44" s="1">
-        <v>-0.19650000000000001</v>
+      <c r="AA44" s="1" t="n">
+        <v>0.1965</v>
       </c>
       <c r="AB44" s="1" t="s">
         <v>227</v>
@@ -5350,6 +5428,11 @@
       </c>
       <c r="AD44" s="1" t="s">
         <v>65</v>
+      </c>
+      <c r="AE44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：已修正。ElHaffar 表1–2（PDF第7页）：交通灯条件高排放菜日销量139低于对照154.875，修正为正向。 原始Cohensd、v及SampleSize保持不变。 沿用当前提取的绝对日销量结局，未改为销量份额。</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -5419,14 +5502,14 @@
       <c r="X45" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="Y45" s="1">
-        <v>1</v>
+      <c r="Y45" s="1" t="n">
+        <v>-1</v>
       </c>
       <c r="Z45" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="AA45" s="1">
-        <v>-0.10249999999999999</v>
+      <c r="AA45" s="1" t="n">
+        <v>0.1025</v>
       </c>
       <c r="AB45" s="1" t="s">
         <v>228</v>
@@ -5436,6 +5519,11 @@
       </c>
       <c r="AD45" s="1" t="s">
         <v>65</v>
+      </c>
+      <c r="AE45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：已修正。ElHaffar 表1–2（PDF第7页）：单一标签条件低排放菜日销量133.750高于对照126.125，修正为正向。 原始Cohensd、v及SampleSize保持不变。 沿用当前提取的绝对日销量结局，未改为销量份额。</t>
+        </is>
       </c>
     </row>
     <row r="46" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -5505,14 +5593,14 @@
       <c r="X46" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="Y46" s="1">
-        <v>-1</v>
+      <c r="Y46" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="Z46" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="AA46" s="1">
-        <v>0.1285</v>
+      <c r="AA46" s="1" t="n">
+        <v>-0.1285</v>
       </c>
       <c r="AB46" s="1" t="s">
         <v>228</v>
@@ -5522,6 +5610,11 @@
       </c>
       <c r="AD46" s="1" t="s">
         <v>65</v>
+      </c>
+      <c r="AE46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：已修正。ElHaffar 表1–2（PDF第7页）：单一标签条件高排放菜日销量170.875高于对照160.500，修正为负向。 原始Cohensd、v及SampleSize保持不变。 沿用当前提取的绝对日销量结局，未改为销量份额。</t>
+        </is>
       </c>
     </row>
     <row r="47" spans="1:30" x14ac:dyDescent="0.2">
@@ -5867,6 +5960,11 @@
       <c r="AD50" s="1" t="s">
         <v>40</v>
       </c>
+      <c r="AE50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28：待处理，数值暂留。Bentil：现有d及v可由受邀样本89/72复现，但该N不是购买结局有效样本。需取得干预后有效n及对应SD/SE。</t>
+        </is>
+      </c>
     </row>
     <row r="51" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
@@ -5893,11 +5991,11 @@
       <c r="H51" s="5">
         <v>54</v>
       </c>
-      <c r="I51" s="6">
-        <v>5.1999999999999998E-3</v>
-      </c>
-      <c r="J51" s="7">
-        <v>302</v>
+      <c r="I51" s="6" t="n">
+        <v>0.527374795144837</v>
+      </c>
+      <c r="J51" s="7" t="n">
+        <v>294</v>
       </c>
       <c r="K51" s="5" t="s">
         <v>47</v>
@@ -5941,17 +6039,23 @@
       <c r="Z51" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="AA51" s="5">
-        <v>5.1999999999999998E-3</v>
+      <c r="AA51" s="5" t="n">
+        <v>0.527374795144837</v>
       </c>
       <c r="AB51" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="AC51" s="5">
-        <v>1.47E-2</v>
+      <c r="AC51" s="5" t="n">
+        <v>0.0156276394721184</v>
       </c>
       <c r="AD51" s="5" t="s">
         <v>40</v>
+      </c>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28 已修正：采用作者排除后数据，每人40轮安全选择的平均比例。干预n=194，共享对照n=100。Cohen’s d=0.527374795145，v=0.015627639472。均值与SD统一为0–1，按参与者而非轮次计算。保留原干预与Control比较及正向编码。Control无实际排放，干预同时引入碳外部性及其信息；此设计属性保留在解释中。两条比较共享同一100人对照。来源：https://osf.io/e78da/；data_study1_clean.RData中的wide_study1.meanChoice_cn。
+历史核查记录（本次已更新数值）：2026-09-28：待处理，数值暂留。Rahmani：比例均值与百分数SD混用可复现现有d及v。最终修正还需锁定排除后的分析样本与对照可比性，未直接放大原d。</t>
+        </is>
       </c>
     </row>
     <row r="52" spans="1:30" x14ac:dyDescent="0.2">
@@ -5979,11 +6083,11 @@
       <c r="H52" s="5">
         <v>55</v>
       </c>
-      <c r="I52" s="6">
-        <v>8.8999999999999999E-3</v>
-      </c>
-      <c r="J52" s="7">
-        <v>303</v>
+      <c r="I52" s="6" t="n">
+        <v>0.916892811681081</v>
+      </c>
+      <c r="J52" s="7" t="n">
+        <v>292</v>
       </c>
       <c r="K52" s="5" t="s">
         <v>47</v>
@@ -6027,17 +6131,23 @@
       <c r="Z52" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="AA52" s="5">
-        <v>8.8999999999999999E-3</v>
+      <c r="AA52" s="5" t="n">
+        <v>0.916892811681081</v>
       </c>
       <c r="AB52" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="AC52" s="5">
-        <v>1.46E-2</v>
+      <c r="AC52" s="5" t="n">
+        <v>0.016647875162293</v>
       </c>
       <c r="AD52" s="5" t="s">
         <v>40</v>
+      </c>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-28 已修正：采用作者排除后数据，每人40轮安全选择的平均比例。干预n=192，共享对照n=100。Cohen’s d=0.916892811681，v=0.016647875162。均值与SD统一为0–1，按参与者而非轮次计算。保留原干预与Control比较及正向编码。Control无实际排放，干预同时引入碳外部性及其信息；此设计属性保留在解释中。两条比较共享同一100人对照。来源：https://osf.io/e78da/；data_study1_clean.RData中的wide_study1.meanChoice_cn。
+历史核查记录（本次已更新数值）：2026-09-28：待处理，数值暂留。Rahmani：比例均值与百分数SD混用可复现现有d及v。最终修正还需锁定排除后的分析样本与对照可比性，未直接放大原d。</t>
+        </is>
       </c>
     </row>
     <row r="53" spans="1:30" x14ac:dyDescent="0.2">

</xml_diff>